<commit_message>
Order 1549: +1 crane day (60.030.0634); add local sync script
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WyD1yjEEVfqqNMkTc2oqqQ
</commit_message>
<xml_diff>
--- a/nta-billing/output/חשבון 7/חשבון 1549 - כהן אלדן.xlsx
+++ b/nta-billing/output/חשבון 7/חשבון 1549 - כהן אלדן.xlsx
@@ -4847,8 +4847,8 @@
         </is>
       </c>
       <c r="D109" s="11">
-        <f>IF(L20&gt;0,IF(SUM(D65,D66,D67,D68,D69,D70)&gt;=5,2,1),0)</f>
-        <v>1</v>
+        <f>IF(L20&gt;0,IF(SUM(D65,D66,D67,D68,D69,D70)&gt;=5,2,1),0)+1</f>
+        <v>2</v>
       </c>
       <c r="E109" s="12" t="n">
         <v>1810</v>
@@ -4867,7 +4867,7 @@
       </c>
       <c r="I109" s="11">
         <f>IF(D109="","",H109*D109)</f>
-        <v>1615.425</v>
+        <v>3230.85</v>
       </c>
     </row>
     <row r="110" hidden="1">
@@ -5557,7 +5557,7 @@
       <c r="H133" s="17" t="n"/>
       <c r="I133" s="19">
         <f>SUMIF(A:A,"60.*",I:I)</f>
-        <v>3146.0625</v>
+        <v>4761.4875</v>
       </c>
     </row>
     <row r="134">
@@ -5611,7 +5611,7 @@
       <c r="H136" s="22" t="n"/>
       <c r="I136" s="22">
         <f>SUM(I125:I135)</f>
-        <v>82703.78287663114</v>
+        <v>84319.20787663115</v>
       </c>
     </row>
     <row r="137">
@@ -5629,7 +5629,7 @@
       <c r="H137" s="22" t="n"/>
       <c r="I137" s="22">
         <f>(I136*(1/100*18))</f>
-        <v>14886.680917793605</v>
+        <v>15177.457417793607</v>
       </c>
     </row>
     <row r="138">
@@ -5647,7 +5647,7 @@
       <c r="H138" s="22" t="n"/>
       <c r="I138" s="22">
         <f>I136+I137</f>
-        <v>97590.46379442475</v>
+        <v>99496.66529442475</v>
       </c>
     </row>
   </sheetData>
@@ -6676,7 +6676,7 @@
       </c>
       <c r="B81" s="32">
         <f>SUM(D84:D86)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C81" s="33" t="inlineStr">
         <is>
@@ -6751,7 +6751,7 @@
       <c r="C85" s="39" t="n"/>
       <c r="D85" s="47">
         <f>IFERROR(INDEX('1549'!D:D,MATCH(A85,'1549'!A:A,0)),0)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E85" s="36" t="inlineStr">
         <is>

</xml_diff>